<commit_message>
Added multi-page pagination support for 100+ listings
</commit_message>
<xml_diff>
--- a/leads.xlsx
+++ b/leads.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,17 +473,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Siemens Industry Software (India) Private Limited</t>
+          <t>X-Plosiv Event &amp; Promotions Pvt. Ltd. - Best Event Company</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -493,17 +493,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Brigade Magnum,B-301, International Airport Road, Amruthahalli- Kodigehalli Gate near, Hebbal, Bengaluru, Karnataka 560048, India</t>
+          <t>714, 718 D Block, Pocket 11, Okhla, New Delhi, Delhi 110025, India</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>+91 1800 202 6796</t>
+          <t>+91 98105 25439</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>http://siemens.com/</t>
+          <t>https://x-plosiv.in/</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -511,17 +511,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Techasoft Pvt. Ltd.</t>
+          <t>SHOWMAKERZ</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3rd Floor, 435, 27th Main Rd, 1st Sector, HSR Layout, Bengaluru, Karnataka 560102, India</t>
+          <t>Building No 31, 4th Floor,, Sant Nagar, East of Kailash, New Delhi, Delhi 110065, India</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>+91 88847 39988</t>
+          <t>+91 98111 73792</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.techasoft.com/</t>
+          <t>https://www.showmakerz.com/</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -549,17 +549,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mindroit Technologies Pvt Ltd</t>
+          <t>Eventales Designs Pvt. Ltd. | Luxury and Corporate Event Management Company in Delhi NCR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -569,39 +569,40 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2nd Floor, Krishna Tower, No: 11, Chandra Layout Main Rd, Income Tax Layout, Binny Mills Employees Colony, Vijayanagar, Bengaluru, Karnataka 560040, India</t>
+          <t>Khasra No. 401, Second Floor, Kaluram Market, Mehrauli-Gurgaon Rd, Ghitorni, New Delhi, Delhi 110030, India</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>+91 78296 52092</t>
+          <t>+91 99100 74464</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>http://www.mindroit.com/</t>
+          <t>https://eventales.com/</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>services@mindroit.com</t>
+          <t xml:space="preserve">hello@eventales.com, hello@eventales.com
+</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Software Company in Bangalore</t>
+          <t>WOW Events Pvt Ltd</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -611,13 +612,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>S End C Cross Rd, KSRTC Layout, 2nd Phase, J. P. Nagar, Bengaluru, Karnataka 560041, India</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>1/7 3rd Floor, WOW Events Pvt. Ltd, above SBI Bank, Block 1, East Patel Nagar, Patel Nagar, New Delhi, Delhi 110008, India</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+91 11 4248 8720</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>http://blogscompass.com/</t>
+          <t>http://www.wowevents.in/</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -625,17 +630,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Object IT Solutions INDIA Pvt. Ltd</t>
+          <t>SOS Party - Offsite Event Management Company Delhi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -645,39 +650,35 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1st Floor, 75/757, 10th Main Rd, 4th Block, Jayanagar, Bengaluru, Karnataka 560011, India</t>
+          <t>Gate no. 2, Metro Station, Ground Floor, N-161, Saira Tower, Marg, near Green Park, Gautam Nagar, New Delhi, Delhi 110049, India</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>+91 94805 29808</t>
+          <t>+91 79734 32360</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>http://www.objectit.com/</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>hr@objectit.com</t>
-        </is>
-      </c>
+          <t>https://www.sosparty.io/</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IFORTIS WORLDWIDE</t>
+          <t>Neer Event Management</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -687,13 +688,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Level 14 &amp; 15, UB City, Concorde Towers, 1, Vittal Mallya Rd, Shanthala Nagar, Ashok Nagar, Bengaluru, Karnataka 560001, India</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>C-1/2, Block D2, Milap Nagar, Uttam Nagar, Delhi, 110059, India</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>+91 89509 19304</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://ifortisworldwide.org/</t>
+          <t>https://www.neereventsmanagement.com/</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -701,17 +706,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Unvired Software India Pvt. Ltd.</t>
+          <t>Theming Ideas - Best Event Management Company In Delhi NCR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -721,39 +726,39 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>No.82, Old No.290/A, 2nd Floor, 9th Main Road, 34th Cross Rd, 4th Block, Jayanagar, Bengaluru, Karnataka 560011, India</t>
+          <t>102, 1st Floor, P Block, Pocket A, Sector 18, Noida, Uttar Pradesh 201301, India</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>+91 7135 602 760</t>
+          <t>+91 98183 35808</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://unvired.com/</t>
+          <t>http://www.themingideas.com/</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>sales@unvired.com</t>
+          <t>ideas@themingideas.com</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Lore Software Solutions Pvt. Ltd.</t>
+          <t>Awesome Event | Best Event Company in Delhi NCR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -763,17 +768,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1, 1st Main, 1st A Cross Rd, Mico Layout, BTM Layout 2nd Stage, BTM Layout, Bengaluru, Karnataka 560076, India</t>
+          <t>street no.12, House no.121b, near Radha Kishan Mandir, Block G, New Delhi, Delhi 110080, India</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>+91 80 4264 5673</t>
+          <t>+91 84477 16668</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.loresoftwaresolutions.com/</t>
+          <t>https://sites.google.com/view/awesomeeventpvtltd/home</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -781,17 +786,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Gadget Software India Private Limited</t>
+          <t>Anandam Events</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -801,17 +806,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14th Cross Road, 1053, 30th Main Rd, Banashankari Stage II, Bengaluru, Karnataka 560070, India</t>
+          <t>First Floor, B-1/3, near Brands Show Sha, B 1 Block, Paschim Vihar, New Delhi, Delhi, 110063, India</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>+91 80 2671 6923</t>
+          <t>+91 98716 67970</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>http://www.gadgetsoftware.com/</t>
+          <t>https://www.anandamevents.com/</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -819,17 +824,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MRI Software India Pvt Ltd</t>
+          <t>SS Events &amp; Co.</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -839,13 +844,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>8th floor, 12, Commerce@Mantri, 1 &amp; 2, Bannerghatta Rd, NS Palya, BTM Layout 2nd Stage, BTM Layout, Bengaluru, Karnataka 560076, India</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>Block G, Kalkaji, New Delhi, Delhi 110019, India</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>+91 99904 95905</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.mrisoftware.com/</t>
+          <t>http://www.sseventsn.com/</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -853,17 +862,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Enverus India Pvt Ltd ( HQ)</t>
+          <t>Loud In Crowd Events</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -873,35 +882,39 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Indiqube, South Summit, 18 &amp; 18/1, Vijayarangam Layout, Jayanagar, Bengaluru, Karnataka 560004, India</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>H. No. 53,54-A, Ground Floor, Dayal Sar Colony SOUTH EXTN PART-III, Uttam Nagar, New Delhi, West, Delhi, 110059, India</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>+91 96437 84717</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.enverus.com//</t>
+          <t>http://www.loudincrowd.com/</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>accountsreceivable@enverus.com, energyanalyticssupport@enverus.com, workbenchsupport@enverus.com, rfxsupport@enverus.com, openinvoicesupport@enverus.com, mineralsoftsupport@enverus.com, powersupport@enverus.com, interconnect@enverus.com, tradingandrisksupport@enverus.com</t>
+          <t>info@loudincrowd.com, Info@loudincrowd.com</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Esi Software India Private Limited</t>
+          <t>Nextera Entertainment</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -911,35 +924,31 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>KALYANI MAGNUM, Krishnaraju Layout, Amalodbhavi Nagar, Panduranga Nagar, Bengaluru, Karnataka 560070, India</t>
+          <t>D-144, 1st Floor, Flat No. B-5, Krishna Park, Khanpur (9863522222), New Delhi, Delhi 110080, India</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>+91 80 4181 8400</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>https://www.esi-group.com/company/worldwide/india</t>
-        </is>
-      </c>
+          <t>+91 98992 91066</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sirius Embedded Software Private Limited</t>
+          <t>Hitkari Productions and Creations | Best Event Planner in Delhi NCR | Best Wedding Planner</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -949,39 +958,39 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3RD FLOOR, WEST INN, INSPIRA, opposite YES BANK, Jayanagar 3rd Block, Bengaluru, Karnataka 560011, India</t>
+          <t>Upper Basement 4, Arunachal Building, Barakhamba Rd, Barakhamba, New Delhi, Delhi 110001, India</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>+91 95133 00147</t>
+          <t>+91 85888 50883</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://excelfore.com/</t>
+          <t>https://hitkariproductions.com/</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>sales@excelfore.com</t>
+          <t>info@hitkariproductions.com</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Trigent Software Pvt. Ltd. - IT Services Division</t>
+          <t>Knight Kings Entertainment Private Limited</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -991,39 +1000,39 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1st Floor, West Wing, Khanija Bhavan, 49, Race Course Rd, Racecourse, Gandhi Nagar, Bengaluru, Karnataka 560001, India</t>
+          <t>103, A/1, Gautam Nagar, New Delhi, Delhi 110049, India</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>+91 80 2226 3000</t>
+          <t>+91 98110 00084</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://trigent.com/?utm_source=GMB-IN&amp;utm_medium=organic&amp;utm_campaign=TrigentHome</t>
+          <t>http://www.knightkings.com/</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>sales@trigent.com</t>
+          <t>info@knightkings.com</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Superior Codelabs - Best Software development company in Bangalore, India</t>
+          <t>Blue Box Events</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1033,17 +1042,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3rd floor, Cunningham Classic, Cunningham Rd, Shivaji Nagar, Bengaluru, Karnataka 560001, India</t>
+          <t>451, Bhai Parmanand Colony, Mukherjee Nagar, New Delhi, Delhi, 110033, India</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>+91 96112 01204</t>
+          <t>+91 97163 22858</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>http://www.superiorcodelabs.com/</t>
+          <t>https://blueboxevents.co.in/</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
@@ -1051,17 +1060,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Zenefits Technologies India Private Limited</t>
+          <t>Celebration Planner - Kids Party Organisers Activity and Decoration In Delhi NCR</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1071,13 +1080,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ward No. 146, #8/2, 2nd Floor, Bren Optimus, C/O TableSpace Office Dr. MH, Marigowda Rd, Adugodi, Bengaluru, Karnataka 560030, India</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>C-2/97, Block C-2, Pocket 2, Sector 16, Rohini, Delhi, 110089, India</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>+91 95607 94830</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>http://www.zenefits.com/</t>
+          <t>https://www.kidspartyorganisers.in/</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -1085,17 +1098,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Checkpoint Systems Software India Pvt Limited</t>
+          <t>Nishant Sharma Events Pvt. Ltd.</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1103,37 +1116,25 @@
           <t>India</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Fernbank, 3, Rest House Rd, Shanthala Nagar, Ashok Nagar, Bengaluru, Karnataka 560001, India</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>+91 80665 95200</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>http://www.checkpointsystems.com/</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>eGenius - ERP Software in Bangalore</t>
+          <t>Big Shot Event Co.</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Software company</t>
+          <t>Event management company</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>bengaluru</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1143,20 +1144,1256 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>No 646/52, 2nd Block, Rajajinagar, Bengaluru, Karnataka 560010, India</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>+91 99869 94328</t>
-        </is>
-      </c>
+          <t>Plot no.10, G/F, Meenakshi Garden, Tilak Nagar, Delhi, 110018, India</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>http://egenius.in/</t>
+          <t>https://bigshotevent.com/</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Floodlightz Events</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Ganesh Das Building, 8555, Roshanara Rd, Sabzi Mandi Old, Delhi, 110007, India</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>+91 97180 76443</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://floodlightz.com/</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>nikhil@floodlightz.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Royal Hub</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Basement (Front Lower Ground Floor, S-473, Greater Kailash - 2, Block S, Greater Kailash II, Greater Kailash, New Delhi, Delhi 110048, India</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>+91 87002 49372</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.royalhub.in/</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Advents Events &amp; Research</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Dharampal Colony, E-111, Ali Vihar, Sarita Vihar, Ali, New Delhi, Delhi 110076, India</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>+91 88267 47278</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>http://www.adventsear.com/</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Acoustic Event &amp; Management Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Madersa Meir, Jumla Street, 1718, Ajmere Gate Rd, Lal Kuan Bazar, Ajmeri Gate, New Delhi, Delhi, 110006, India</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>+91 98916 44064</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>http://acousticpvtltd.com/</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Narayan Events Management</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Advertising agency</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>245-B, Sant Nagar, East of Kailash, New Delhi, Delhi 110065, India</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>+91 72988 88891</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Namah India</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>3/9 Basement, Block 6, East Patel Nagar, Patel Nagar, New Delhi, Delhi 110008, India</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>+91 98598 51030</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>http://www.namahindia.com/</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Info@namahindia.com,  Info@namahindia.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>The Chopra Events Group</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>25/377, Block B, New Moti Nagar, Moti Nagar, New Delhi, Delhi, 110015, India</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>+91 82852 53313</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Katalyst Entertainment Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>198, 2nd Floor Opposite, Sapna Cinema Road, 14, Ramesh Market, East of Kailash, New Delhi, Delhi 110065, India</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>+91 98998 85522</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.katalystworld.com/</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>connect@katalystworld.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ANBC Events</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>E-261, Block E, Lajpat Nagar IV, Lajpat Nagar, New Delhi, Delhi 110024, India</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>+91 88000 00142</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>http://www.anbcevents.com/</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>info@anbcevents.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Crew4Events</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Third Floor, E-10, South Extension II, New Delhi, Delhi 110049, India</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>+91 96502 41114</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>http://crew4events.com/</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>info@crew4events.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Wizard Events &amp; Conferences Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>203, SURYA KIRAN BUILDING, KG Marg, Atul Grove Road, Janpath, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>+91 93105 02495</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.wizard-events.in/</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>info@wizard-events.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SL Entertainment &amp; Events - best event management company in Delhi | corporate event Planners | Celebrity booking</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Ansal Complex, B-516, 2, Bhikaji Cama Place, Rama Krishna Puram, New Delhi, Delhi 110066, India</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://slentertainment.in/</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Svg Broad Media Event Management Company (Svg Events Pvt. Ltd.)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Main Market, Narwana Rd, Vinod Nagar North, Ambedkar Park, Patparganj, Mandawali, Delhi, 110092, India</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>+91 98119 21126</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://svg-broad-media-event.grexa.site/</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Spectrum Events</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Second Floor, FIEE Complex, A56, Block A, Okhla Phase II, Okhla Industrial Estate, New Delhi, Delhi 110020, India</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>+91 11 4500 6347</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://spectrumevents.in/</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>contact@spectrumevents.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Primar Partners - BTL &amp; MICE Agency</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>UGF, Lane No-2, B15/292, Westend Marg, Saidulajab, Saiyad Ul Ajaib Village, Sainik Farm, New Delhi, Delhi 110030, India</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>+91 98117 31411</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.primarpartners.in/</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>info@primarpartners.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Pearl Imagica - Event Management, Corporate Events in Delhi</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Ashok Vihar Phase 1 Rd, Pocket H, Phase 1, Ashok Vihar, New Delhi, Delhi, 110052, India</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>+91 93150 62160</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>http://www.pearlimagica.com/</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>The Silver Stage - Event Management Company</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>B, 3rd floor, LIG Flats, L1/281, Block L 1, Kalkaji, New Delhi, Delhi 110019, India</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>+91 99909 06777</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>http://thesilverstage.com/</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>info@thesilverstage.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>A1 Event Solutions</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Block B-1, A-24/9, Mathura Rd, Mohan Cooperative Industrial Estate, Saidabad, New Delhi, Delhi 110044, India</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>+91 84473 00532</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>http://a1eventsolutions.in/</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Manish@a1eventsolutions.in, info@a1eventsolutions.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>ShowTime Event - Corporate Event Planner, Artist management Company</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>3rd Floor, A- 50 &amp; 51, Prem Nagar, Block E, Param Puri, Uttam Nagar, Delhi, 110059, India</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>+91 98710 09325</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.showtimeevent.com/</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>info@showtimeevent.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>TEC INDIA ENTERTAINMENT PVT.LTD</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Savitri Cinema Complex, Inder Mohan Bhardwaj Marg, Block E, Greater Kailash II, Greater Kailash, New Delhi, Delhi 110048, India</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>http://tecindia.in/</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>TAFCON Projects (India) Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>9th Floor, Devika Tower, 923 &amp; 923A, 6, Nehru Place, New Delhi, Delhi 110019, India</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>+91 11 4985 7777</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://tafcon.in/</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>events@tafcon.in</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>SKY Events India (Corporate Events &amp; Celebrity Artists Management)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>D 107, D Block, Sector 2, Noida, Uttar Pradesh 201301, India</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>+91 99118 15599</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>http://www.skyevents.in/</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>APSG Events| Destination Wedding Planner| Corporate Event Management Company in New Delhi</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Block E, Malviya Nagar, New Delhi, Delhi 110017, India</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>+91 93152 99416</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.apsgevents.com/</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>info@apsgevents.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Limelight Events - Best Corporate Event Management Company in Delhi NCR</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>3,4, Building 1, A-13/2, Highway Towers, BC-14, Lotus Boulevard, Sector 100, Noida, Uttar Pradesh 201309, India</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>+91 81308 77300</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.limelightevents.in/</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Effortless Events Pvt.ltd</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>+91 78380 08069</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://effortlessevents.in/</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>7WD Wedding Planner &amp; Event Management</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>7WD Wedding Planner &amp; Event Management 7 WONDERS DESIGNING INSTITUTIONS PRIVATE LIMITED Place L29 - L34, First Floor, Awfis Building, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Tritya Institute of Event Management - TIEM DELHI - Best Event Management Institute in Delhi</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>College</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>NO. 2, G - 5, 2ND &amp; 3RD FLOOR SOUTH EXTENSION PART -1, opp. SOUTH EX METRO GATE, above CROCS SHOWROOM, Main Market, New Delhi, Delhi 110049, India</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>+91 99909 37354</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>http://www.tiemdelhi.com/</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>admissions@tiemdelhi.com, placements@tiemdelhi.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>P&amp;M Events</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>D Block, Pocket D, Rajender Nagar Part 1, New Rajinder Nagar, New Delhi, Delhi, 110060, India</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>+91 77770 00038</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CRI Events Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2nd &amp; 3rd Floor, 13/4, West Patel Nagar, Block 13, West Patel Nagar, New Delhi, Delhi 110008, India</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>+91 11 6450 0178</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>http://www.crievents.com/</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Shaandaar Events - Best Destination Wedding Planner in Delhi</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>First Floor, Awfis Co-working, Hanuman Road Area, Connaught Place, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>+91 70189 02594</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://shaandaarevents.com/wedding-planner-in-delhi-ncr/</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Craftworld Events</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Event management company</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>52/20, 1st Floor, Ramjas Road, Karol Bagh, New Delhi, Delhi 110005, India</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>+91 98203 44426</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>http://craftworldevents.com/corporate-event-management-company-delhi-ncr-gurgaon/</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DC Wedding And Events</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Event planner</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>69, Regal Building, Connaught Cir, Hanuman Road Area, Connaught Place, Delhi, New Delhi, Delhi 110001, India</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>+91 99991 10651</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://www.dcweddingandevents.com/</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>